<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-11
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-10" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-11" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -95,38 +95,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Amgen</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Biostatistics Senior Manager, Biosimilars US- Remote</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">United States - Remote</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Posted Yesterday</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://amgen.wd1.myworkdayjobs.com/job/United-States---Remote/Biostatistics-Senior-Manager--Biosimilars-US--Remote_R-242819</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workday</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-14
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-13" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-14" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -95,6 +95,38 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associate Director, Real World Biostatistics</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USA - Pennsylvania - Upper Providence</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posted Today</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://gsk.wd5.myworkdayjobs.com/job/USA---Pennsylvania---Upper-Providence/Associate-Director--Real-World-Biostatistics_447563</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workday</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-15
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-14" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-15" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -113,7 +113,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted Today</t>
+          <t xml:space="preserve">Posted Yesterday</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-16
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-15" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-16" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -98,17 +98,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSK</t>
+          <t xml:space="preserve">Gilead Sciences</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Associate Director, Real World Biostatistics</t>
+          <t xml:space="preserve">Sr Manager, Biostatistics</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">USA - Pennsylvania - Upper Providence</t>
+          <t xml:space="preserve">United States - California - Foster City</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -118,7 +118,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://gsk.wd5.myworkdayjobs.com/job/USA---Pennsylvania---Upper-Providence/Associate-Director--Real-World-Biostatistics_447563</t>
+          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Sr-Manager--Biostatistics_R0055822-3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-17
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-16" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-17" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -103,12 +103,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr Manager, Biostatistics</t>
+          <t xml:space="preserve">Associate Director, Biostatistics- Virology</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States - California - Foster City</t>
+          <t xml:space="preserve">2 Locations</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -118,7 +118,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Sr-Manager--Biostatistics_R0055822-3</t>
+          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Associate-Director--Biostatistics--Virology_R0055850-2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-18
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-17" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-18" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -95,38 +95,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gilead Sciences</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Associate Director, Biostatistics- Virology</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 Locations</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Posted Yesterday</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Associate-Director--Biostatistics--Virology_R0055850-2</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workday</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-27
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-26" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-27" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -95,6 +95,38 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSK</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associate Director - Oncology Statistics</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Locations</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posted Today</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://gsk.wd5.myworkdayjobs.com/job/UK--London--New-Oxford-Street/Associate-Director---Oncology-Statistics_450338-1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workday</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
 </worksheet>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-28
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-27" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-28" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -98,17 +98,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSK</t>
+          <t xml:space="preserve">AstraZeneca</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Associate Director - Oncology Statistics</t>
+          <t xml:space="preserve">Statistical Programming Associate Director</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 Locations</t>
+          <t xml:space="preserve">US - Durham - NC</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -118,10 +118,42 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t xml:space="preserve">https://astrazeneca.wd3.myworkdayjobs.com/job/US---Durham---NC/Statistical-Programming-Associate-Director_R-262991</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workday</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associate Director - Oncology Statistics</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 Locations</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posted Yesterday</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t xml:space="preserve">https://gsk.wd5.myworkdayjobs.com/job/UK--London--New-Oxford-Street/Associate-Director---Oncology-Statistics_450338-1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t xml:space="preserve">workday</t>
         </is>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-29
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-28" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-29" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -98,27 +98,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">AstraZeneca</t>
+          <t xml:space="preserve">Gilead Sciences</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Statistical Programming Associate Director</t>
+          <t xml:space="preserve">Sr Manager, Biostatistics</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">US - Durham - NC</t>
+          <t xml:space="preserve">United States - California - Foster City</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Posted Today</t>
+          <t xml:space="preserve">Posted Yesterday</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://astrazeneca.wd3.myworkdayjobs.com/job/US---Durham---NC/Statistical-Programming-Associate-Director_R-262991</t>
+          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Sr-Manager--Biostatistics_R0055822-3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -130,17 +130,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSK</t>
+          <t xml:space="preserve">AstraZeneca</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Associate Director - Oncology Statistics</t>
+          <t xml:space="preserve">Statistical Programming Associate Director</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 Locations</t>
+          <t xml:space="preserve">US - Durham - NC</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -150,10 +150,42 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://gsk.wd5.myworkdayjobs.com/job/UK--London--New-Oxford-Street/Associate-Director---Oncology-Statistics_450338-1</t>
+          <t xml:space="preserve">https://astrazeneca.wd3.myworkdayjobs.com/job/US---Durham---NC/Statistical-Programming-Associate-Director_R-262991</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">workday</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSL Behring</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associate Director, Biostatistics</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 Locations</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Posted Today</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://csl.wd1.myworkdayjobs.com/job/Americas-US-PA-King-of-Prussia-CSL-Behring/Principal-Statistician_R-282817</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">workday</t>
         </is>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-30
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-29" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-30" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -98,17 +98,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gilead Sciences</t>
+          <t xml:space="preserve">CSL Behring</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sr Manager, Biostatistics</t>
+          <t xml:space="preserve">Associate Director, Biostatistics</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">United States - California - Foster City</t>
+          <t xml:space="preserve">5 Locations</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -118,74 +118,10 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://gilead.wd1.myworkdayjobs.com/job/United-States---California---Foster-City/Sr-Manager--Biostatistics_R0055822-3</t>
+          <t xml:space="preserve">https://csl.wd1.myworkdayjobs.com/job/Americas-US-PA-King-of-Prussia-CSL-Behring/Principal-Statistician_R-282817</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workday</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">AstraZeneca</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Statistical Programming Associate Director</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">US - Durham - NC</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Posted Yesterday</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://astrazeneca.wd3.myworkdayjobs.com/job/US---Durham---NC/Statistical-Programming-Associate-Director_R-262991</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workday</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CSL Behring</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Associate Director, Biostatistics</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Locations</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Posted Today</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://csl.wd1.myworkdayjobs.com/job/Americas-US-PA-King-of-Prussia-CSL-Behring/Principal-Statistician_R-282817</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
         <is>
           <t xml:space="preserve">workday</t>
         </is>

</xml_diff>

<commit_message>
daily-jobs: biostat SM/AD scrape for 2026-10-31
</commit_message>
<xml_diff>
--- a/daily-jobs/latest.xlsx
+++ b/daily-jobs/latest.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="24h jobs 2026-10-30" sheetId="1" r:id="rId1"/>
+    <sheet name="24h jobs 2026-10-31" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -95,38 +95,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CSL Behring</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Associate Director, Biostatistics</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 Locations</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Posted Yesterday</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://csl.wd1.myworkdayjobs.com/job/Americas-US-PA-King-of-Prussia-CSL-Behring/Principal-Statistician_R-282817</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">workday</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
 </worksheet>

</xml_diff>